<commit_message>
score, pause et recommencer et rapport
</commit_message>
<xml_diff>
--- a/doc/P-BULL-DEV-RayanSahbani-jnltrav.xlsx
+++ b/doc/P-BULL-DEV-RayanSahbani-jnltrav.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="30430"/>
   <workbookPr updateLinks="never" codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ETMLFID2\Projet\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\ETMLFID2\Projet\p-bulle-snake-step1-start\P_BULL_DEV_SNAKE\doc\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D97CBDD-EB8D-4F95-AF9C-1702663F20B7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB29226A-A4B2-4BBC-8AF7-488BFCBDBA38}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-27675" yWindow="1125" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Journal" sheetId="18" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="29">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="72" uniqueCount="40">
   <si>
     <t>Apprenti.e</t>
   </si>
@@ -137,6 +137,39 @@
   </si>
   <si>
     <t>absent</t>
+  </si>
+  <si>
+    <t>Correction de la structure du projet (fichiers dans src/) et ajout des export manquants</t>
+  </si>
+  <si>
+    <t>Génération et affichage de la nourriture (generateFood, drawFood)</t>
+  </si>
+  <si>
+    <t>Affichage du serpent sur le canevas (drawSnake)</t>
+  </si>
+  <si>
+    <t>férié</t>
+  </si>
+  <si>
+    <t>Jour férié</t>
+  </si>
+  <si>
+    <t>Gestion de l'alimentation : le serpent grandit en mangeant la nourriture</t>
+  </si>
+  <si>
+    <t>Gestion des collisions avec les murs (checkWallCollision)</t>
+  </si>
+  <si>
+    <t>Gestion des collisions avec le corps du serpent (checkCollision)</t>
+  </si>
+  <si>
+    <t>Affichage et incrémentation du score</t>
+  </si>
+  <si>
+    <t>Pause et reprise du jeu avec la touche Espace et ajout du choix rejouer / quitter en fin de partie</t>
+  </si>
+  <si>
+    <t>rapport</t>
   </si>
 </sst>
 </file>
@@ -481,18 +514,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
     <xf numFmtId="14" fontId="3" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
       <protection locked="0"/>
@@ -510,6 +531,18 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="3">
@@ -844,10 +877,10 @@
       <c r="A1" s="19" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="28" t="s">
+      <c r="B1" s="33" t="s">
         <v>18</v>
       </c>
-      <c r="C1" s="28"/>
+      <c r="C1" s="33"/>
       <c r="D1" s="20" t="s">
         <v>1</v>
       </c>
@@ -859,10 +892,10 @@
       <c r="A2" s="19" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="28" t="s">
+      <c r="B2" s="33" t="s">
         <v>22</v>
       </c>
-      <c r="C2" s="28"/>
+      <c r="C2" s="33"/>
       <c r="D2" s="20" t="s">
         <v>3</v>
       </c>
@@ -874,10 +907,10 @@
       <c r="A3" s="19" t="s">
         <v>5</v>
       </c>
-      <c r="B3" s="28" t="s">
+      <c r="B3" s="33" t="s">
         <v>20</v>
       </c>
-      <c r="C3" s="28"/>
+      <c r="C3" s="33"/>
       <c r="D3" s="20" t="s">
         <v>6</v>
       </c>
@@ -889,12 +922,12 @@
       <c r="A4" s="19" t="s">
         <v>7</v>
       </c>
-      <c r="B4" s="29" t="s">
+      <c r="B4" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="C4" s="30"/>
-      <c r="D4" s="30"/>
-      <c r="E4" s="31"/>
+      <c r="C4" s="35"/>
+      <c r="D4" s="35"/>
+      <c r="E4" s="36"/>
     </row>
     <row r="5" spans="1:5" ht="21" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
@@ -915,35 +948,35 @@
     </row>
     <row r="6" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4"/>
-      <c r="B6" s="32"/>
+      <c r="B6" s="28"/>
       <c r="C6" s="5"/>
       <c r="D6" s="6"/>
       <c r="E6" s="21"/>
     </row>
     <row r="7" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7"/>
-      <c r="B7" s="33"/>
+      <c r="B7" s="29"/>
       <c r="C7" s="8"/>
       <c r="D7" s="9"/>
       <c r="E7" s="8"/>
     </row>
     <row r="8" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7"/>
-      <c r="B8" s="33"/>
+      <c r="B8" s="29"/>
       <c r="C8" s="8"/>
       <c r="D8" s="9"/>
       <c r="E8" s="8"/>
     </row>
     <row r="9" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7"/>
-      <c r="B9" s="33"/>
+      <c r="B9" s="29"/>
       <c r="C9" s="8"/>
       <c r="D9" s="9"/>
       <c r="E9" s="8"/>
     </row>
     <row r="10" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="10"/>
-      <c r="B10" s="33"/>
+      <c r="B10" s="29"/>
       <c r="C10" s="10"/>
       <c r="D10" s="11"/>
       <c r="E10" s="10"/>
@@ -952,7 +985,7 @@
       <c r="A11" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="33"/>
+      <c r="B11" s="29"/>
       <c r="C11" s="22">
         <f>SUM(C6:C10)</f>
         <v>0</v>
@@ -964,7 +997,7 @@
       <c r="A12" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B12" s="34"/>
+      <c r="B12" s="30"/>
       <c r="C12" s="25"/>
       <c r="D12" s="26"/>
       <c r="E12" s="27"/>
@@ -973,7 +1006,7 @@
       <c r="A13" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="B13" s="32">
+      <c r="B13" s="28">
         <v>46265</v>
       </c>
       <c r="C13" s="5">
@@ -988,7 +1021,7 @@
       <c r="A14" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="33"/>
+      <c r="B14" s="29"/>
       <c r="C14" s="8">
         <v>4</v>
       </c>
@@ -1001,7 +1034,7 @@
       <c r="A15" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="B15" s="33"/>
+      <c r="B15" s="29"/>
       <c r="C15" s="8">
         <v>4</v>
       </c>
@@ -1012,14 +1045,14 @@
     </row>
     <row r="16" spans="1:5" ht="38.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7"/>
-      <c r="B16" s="33"/>
+      <c r="B16" s="29"/>
       <c r="C16" s="8"/>
       <c r="D16" s="9"/>
       <c r="E16" s="8"/>
     </row>
     <row r="17" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="10"/>
-      <c r="B17" s="33"/>
+      <c r="B17" s="29"/>
       <c r="C17" s="10"/>
       <c r="D17" s="11"/>
       <c r="E17" s="10"/>
@@ -1028,7 +1061,7 @@
       <c r="A18" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B18" s="33"/>
+      <c r="B18" s="29"/>
       <c r="C18" s="22">
         <f>SUM(C13:C17)</f>
         <v>12</v>
@@ -1040,7 +1073,7 @@
       <c r="A19" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B19" s="34"/>
+      <c r="B19" s="30"/>
       <c r="C19" s="25"/>
       <c r="D19" s="26"/>
       <c r="E19" s="27"/>
@@ -1049,7 +1082,7 @@
       <c r="A20" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="B20" s="32">
+      <c r="B20" s="28">
         <v>46272</v>
       </c>
       <c r="C20" s="5">
@@ -1062,28 +1095,28 @@
     </row>
     <row r="21" spans="1:5" ht="26.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7"/>
-      <c r="B21" s="33"/>
+      <c r="B21" s="29"/>
       <c r="C21" s="8"/>
       <c r="D21" s="9"/>
       <c r="E21" s="8"/>
     </row>
     <row r="22" spans="1:5" ht="48" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7"/>
-      <c r="B22" s="33"/>
+      <c r="B22" s="29"/>
       <c r="C22" s="8"/>
       <c r="D22" s="9"/>
       <c r="E22" s="8"/>
     </row>
     <row r="23" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7"/>
-      <c r="B23" s="33"/>
+      <c r="B23" s="29"/>
       <c r="C23" s="8"/>
       <c r="D23" s="9"/>
       <c r="E23" s="8"/>
     </row>
     <row r="24" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A24" s="10"/>
-      <c r="B24" s="33"/>
+      <c r="B24" s="29"/>
       <c r="C24" s="10"/>
       <c r="D24" s="11"/>
       <c r="E24" s="10"/>
@@ -1092,7 +1125,7 @@
       <c r="A25" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B25" s="33"/>
+      <c r="B25" s="29"/>
       <c r="C25" s="22">
         <f>SUM(C20:C24)</f>
         <v>12</v>
@@ -1104,42 +1137,62 @@
       <c r="A26" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B26" s="34"/>
+      <c r="B26" s="30"/>
       <c r="C26" s="25"/>
       <c r="D26" s="26"/>
       <c r="E26" s="27"/>
     </row>
     <row r="27" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="4"/>
-      <c r="B27" s="32"/>
-      <c r="C27" s="5"/>
-      <c r="D27" s="6"/>
+      <c r="A27" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B27" s="28">
+        <v>44088</v>
+      </c>
+      <c r="C27" s="5">
+        <v>4</v>
+      </c>
+      <c r="D27" t="s">
+        <v>29</v>
+      </c>
       <c r="E27" s="21"/>
     </row>
     <row r="28" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A28" s="4"/>
-      <c r="B28" s="33"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="9"/>
+      <c r="A28" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B28" s="29"/>
+      <c r="C28" s="8">
+        <v>4</v>
+      </c>
+      <c r="D28" t="s">
+        <v>30</v>
+      </c>
       <c r="E28" s="8"/>
     </row>
     <row r="29" spans="1:5" ht="33" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="4"/>
-      <c r="B29" s="33"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="9"/>
+      <c r="A29" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B29" s="29"/>
+      <c r="C29" s="8">
+        <v>4</v>
+      </c>
+      <c r="D29" t="s">
+        <v>31</v>
+      </c>
       <c r="E29" s="8"/>
     </row>
     <row r="30" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="7"/>
-      <c r="B30" s="33"/>
+      <c r="B30" s="29"/>
       <c r="C30" s="8"/>
       <c r="D30" s="9"/>
       <c r="E30" s="8"/>
     </row>
     <row r="31" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A31" s="10"/>
-      <c r="B31" s="33"/>
+      <c r="B31" s="29"/>
       <c r="C31" s="10"/>
       <c r="D31" s="11"/>
       <c r="E31" s="10"/>
@@ -1148,10 +1201,10 @@
       <c r="A32" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B32" s="33"/>
+      <c r="B32" s="29"/>
       <c r="C32" s="22">
         <f>SUM(C27:C31)</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D32" s="23"/>
       <c r="E32" s="24"/>
@@ -1160,42 +1213,50 @@
       <c r="A33" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B33" s="34"/>
+      <c r="B33" s="30"/>
       <c r="C33" s="25"/>
       <c r="D33" s="26"/>
       <c r="E33" s="27"/>
     </row>
     <row r="34" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="4"/>
-      <c r="B34" s="32"/>
-      <c r="C34" s="5"/>
-      <c r="D34" s="6"/>
+      <c r="A34" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B34" s="28">
+        <v>46286</v>
+      </c>
+      <c r="C34" s="5">
+        <v>12</v>
+      </c>
+      <c r="D34" t="s">
+        <v>33</v>
+      </c>
       <c r="E34" s="21"/>
     </row>
     <row r="35" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="7"/>
-      <c r="B35" s="33"/>
+      <c r="B35" s="29"/>
       <c r="C35" s="8"/>
       <c r="D35" s="9"/>
       <c r="E35" s="8"/>
     </row>
     <row r="36" spans="1:5" ht="39.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="7"/>
-      <c r="B36" s="33"/>
+      <c r="B36" s="29"/>
       <c r="C36" s="8"/>
       <c r="D36" s="9"/>
       <c r="E36" s="8"/>
     </row>
     <row r="37" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7"/>
-      <c r="B37" s="33"/>
+      <c r="B37" s="29"/>
       <c r="C37" s="8"/>
       <c r="D37" s="9"/>
       <c r="E37" s="8"/>
     </row>
     <row r="38" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A38" s="10"/>
-      <c r="B38" s="33"/>
+      <c r="B38" s="29"/>
       <c r="C38" s="10"/>
       <c r="D38" s="11"/>
       <c r="E38" s="10"/>
@@ -1204,10 +1265,10 @@
       <c r="A39" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B39" s="33"/>
+      <c r="B39" s="29"/>
       <c r="C39" s="22">
         <f>SUM(C34:C38)</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D39" s="23"/>
       <c r="E39" s="24"/>
@@ -1216,42 +1277,62 @@
       <c r="A40" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B40" s="34"/>
+      <c r="B40" s="30"/>
       <c r="C40" s="25"/>
       <c r="D40" s="26"/>
       <c r="E40" s="27"/>
     </row>
     <row r="41" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="4"/>
-      <c r="B41" s="32"/>
-      <c r="C41" s="5"/>
-      <c r="D41" s="6"/>
+      <c r="A41" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B41" s="28">
+        <v>46293</v>
+      </c>
+      <c r="C41" s="5">
+        <v>4</v>
+      </c>
+      <c r="D41" t="s">
+        <v>34</v>
+      </c>
       <c r="E41" s="21"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="7"/>
-      <c r="B42" s="33"/>
-      <c r="C42" s="8"/>
-      <c r="D42" s="9"/>
+      <c r="A42" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B42" s="29"/>
+      <c r="C42" s="8">
+        <v>4</v>
+      </c>
+      <c r="D42" t="s">
+        <v>35</v>
+      </c>
       <c r="E42" s="8"/>
     </row>
     <row r="43" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A43" s="7"/>
-      <c r="B43" s="33"/>
-      <c r="C43" s="8"/>
-      <c r="D43" s="9"/>
+      <c r="A43" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B43" s="29"/>
+      <c r="C43" s="8">
+        <v>4</v>
+      </c>
+      <c r="D43" t="s">
+        <v>36</v>
+      </c>
       <c r="E43" s="8"/>
     </row>
     <row r="44" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="7"/>
-      <c r="B44" s="33"/>
+      <c r="B44" s="29"/>
       <c r="C44" s="8"/>
       <c r="D44" s="9"/>
       <c r="E44" s="8"/>
     </row>
     <row r="45" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A45" s="10"/>
-      <c r="B45" s="33"/>
+      <c r="B45" s="29"/>
       <c r="C45" s="10"/>
       <c r="D45" s="11"/>
       <c r="E45" s="10"/>
@@ -1260,10 +1341,10 @@
       <c r="A46" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B46" s="33"/>
+      <c r="B46" s="29"/>
       <c r="C46" s="22">
         <f>SUM(C41:C45)</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D46" s="23"/>
       <c r="E46" s="24"/>
@@ -1272,42 +1353,60 @@
       <c r="A47" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B47" s="34"/>
+      <c r="B47" s="30"/>
       <c r="C47" s="25"/>
       <c r="D47" s="26"/>
       <c r="E47" s="27"/>
     </row>
     <row r="48" spans="1:5" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A48" s="4"/>
-      <c r="B48" s="32"/>
-      <c r="C48" s="5"/>
-      <c r="D48" s="6"/>
+      <c r="A48" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B48" s="28">
+        <v>46300</v>
+      </c>
+      <c r="C48" s="5">
+        <v>4</v>
+      </c>
+      <c r="D48" t="s">
+        <v>37</v>
+      </c>
       <c r="E48" s="21"/>
     </row>
     <row r="49" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="7"/>
-      <c r="B49" s="33"/>
-      <c r="C49" s="8"/>
-      <c r="D49" s="9"/>
+      <c r="A49" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B49" s="29"/>
+      <c r="C49" s="8">
+        <v>4</v>
+      </c>
+      <c r="D49" t="s">
+        <v>38</v>
+      </c>
       <c r="E49" s="8"/>
     </row>
     <row r="50" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7"/>
-      <c r="B50" s="33"/>
-      <c r="C50" s="8"/>
-      <c r="D50" s="9"/>
+      <c r="B50" s="29"/>
+      <c r="C50" s="8">
+        <v>4</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>39</v>
+      </c>
       <c r="E50" s="8"/>
     </row>
     <row r="51" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="7"/>
-      <c r="B51" s="33"/>
+      <c r="B51" s="29"/>
       <c r="C51" s="8"/>
       <c r="D51" s="9"/>
       <c r="E51" s="8"/>
     </row>
     <row r="52" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A52" s="10"/>
-      <c r="B52" s="33"/>
+      <c r="B52" s="29"/>
       <c r="C52" s="10"/>
       <c r="D52" s="11"/>
       <c r="E52" s="10"/>
@@ -1316,10 +1415,10 @@
       <c r="A53" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B53" s="33"/>
+      <c r="B53" s="29"/>
       <c r="C53" s="22">
         <f>SUM(C48:C52)</f>
-        <v>0</v>
+        <v>12</v>
       </c>
       <c r="D53" s="23"/>
       <c r="E53" s="24"/>
@@ -1328,42 +1427,42 @@
       <c r="A54" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B54" s="34"/>
+      <c r="B54" s="30"/>
       <c r="C54" s="25"/>
       <c r="D54" s="26"/>
       <c r="E54" s="27"/>
     </row>
     <row r="55" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4"/>
-      <c r="B55" s="32"/>
+      <c r="B55" s="28"/>
       <c r="C55" s="5"/>
       <c r="D55" s="6"/>
       <c r="E55" s="21"/>
     </row>
     <row r="56" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="7"/>
-      <c r="B56" s="33"/>
+      <c r="B56" s="29"/>
       <c r="C56" s="8"/>
       <c r="D56" s="9"/>
       <c r="E56" s="8"/>
     </row>
     <row r="57" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="7"/>
-      <c r="B57" s="33"/>
+      <c r="B57" s="29"/>
       <c r="C57" s="8"/>
       <c r="D57" s="9"/>
       <c r="E57" s="8"/>
     </row>
     <row r="58" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7"/>
-      <c r="B58" s="33"/>
+      <c r="B58" s="29"/>
       <c r="C58" s="8"/>
       <c r="D58" s="9"/>
       <c r="E58" s="8"/>
     </row>
     <row r="59" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A59" s="10"/>
-      <c r="B59" s="33"/>
+      <c r="B59" s="29"/>
       <c r="C59" s="10"/>
       <c r="D59" s="11"/>
       <c r="E59" s="10"/>
@@ -1372,7 +1471,7 @@
       <c r="A60" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B60" s="33"/>
+      <c r="B60" s="29"/>
       <c r="C60" s="22">
         <f>SUM(C55:C59)</f>
         <v>0</v>
@@ -1384,42 +1483,42 @@
       <c r="A61" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B61" s="34"/>
+      <c r="B61" s="30"/>
       <c r="C61" s="25"/>
       <c r="D61" s="26"/>
       <c r="E61" s="27"/>
     </row>
     <row r="62" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="4"/>
-      <c r="B62" s="32"/>
+      <c r="B62" s="28"/>
       <c r="C62" s="5"/>
       <c r="D62" s="6"/>
       <c r="E62" s="21"/>
     </row>
     <row r="63" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="7"/>
-      <c r="B63" s="33"/>
+      <c r="B63" s="29"/>
       <c r="C63" s="8"/>
       <c r="D63" s="9"/>
       <c r="E63" s="8"/>
     </row>
     <row r="64" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="7"/>
-      <c r="B64" s="33"/>
+      <c r="B64" s="29"/>
       <c r="C64" s="8"/>
       <c r="D64" s="9"/>
       <c r="E64" s="8"/>
     </row>
     <row r="65" spans="1:5" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="7"/>
-      <c r="B65" s="33"/>
+      <c r="B65" s="29"/>
       <c r="C65" s="8"/>
       <c r="D65" s="9"/>
       <c r="E65" s="8"/>
     </row>
     <row r="66" spans="1:5" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="10"/>
-      <c r="B66" s="33"/>
+      <c r="B66" s="29"/>
       <c r="C66" s="10"/>
       <c r="D66" s="11"/>
       <c r="E66" s="10"/>
@@ -1428,7 +1527,7 @@
       <c r="A67" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B67" s="33"/>
+      <c r="B67" s="29"/>
       <c r="C67" s="22">
         <f>SUM(C62:C66)</f>
         <v>0</v>
@@ -1440,42 +1539,42 @@
       <c r="A68" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B68" s="34"/>
+      <c r="B68" s="30"/>
       <c r="C68" s="25"/>
       <c r="D68" s="26"/>
       <c r="E68" s="27"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A69" s="4"/>
-      <c r="B69" s="32"/>
+      <c r="B69" s="28"/>
       <c r="C69" s="5"/>
       <c r="D69" s="6"/>
       <c r="E69" s="21"/>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A70" s="7"/>
-      <c r="B70" s="33"/>
+      <c r="B70" s="29"/>
       <c r="C70" s="8"/>
       <c r="D70" s="9"/>
       <c r="E70" s="8"/>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A71" s="7"/>
-      <c r="B71" s="33"/>
+      <c r="B71" s="29"/>
       <c r="C71" s="8"/>
       <c r="D71" s="9"/>
       <c r="E71" s="8"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A72" s="7"/>
-      <c r="B72" s="33"/>
+      <c r="B72" s="29"/>
       <c r="C72" s="8"/>
       <c r="D72" s="9"/>
       <c r="E72" s="8"/>
     </row>
     <row r="73" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A73" s="10"/>
-      <c r="B73" s="33"/>
+      <c r="B73" s="29"/>
       <c r="C73" s="10"/>
       <c r="D73" s="11"/>
       <c r="E73" s="10"/>
@@ -1484,7 +1583,7 @@
       <c r="A74" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B74" s="33"/>
+      <c r="B74" s="29"/>
       <c r="C74" s="22">
         <f>SUM(C69:C73)</f>
         <v>0</v>
@@ -1496,41 +1595,41 @@
       <c r="A75" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B75" s="34"/>
+      <c r="B75" s="30"/>
       <c r="C75" s="25"/>
       <c r="D75" s="26"/>
       <c r="E75" s="27"/>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A76" s="4"/>
-      <c r="B76" s="32"/>
+      <c r="B76" s="28"/>
       <c r="C76" s="5"/>
       <c r="D76" s="9"/>
       <c r="E76" s="21"/>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A77" s="7"/>
-      <c r="B77" s="33"/>
+      <c r="B77" s="29"/>
       <c r="C77" s="8"/>
       <c r="E77" s="8"/>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A78" s="7"/>
-      <c r="B78" s="33"/>
+      <c r="B78" s="29"/>
       <c r="C78" s="8"/>
       <c r="D78" s="9"/>
       <c r="E78" s="8"/>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A79" s="7"/>
-      <c r="B79" s="33"/>
+      <c r="B79" s="29"/>
       <c r="C79" s="8"/>
       <c r="D79" s="9"/>
       <c r="E79" s="8"/>
     </row>
     <row r="80" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="10"/>
-      <c r="B80" s="33"/>
+      <c r="B80" s="29"/>
       <c r="C80" s="10"/>
       <c r="D80" s="11"/>
       <c r="E80" s="10"/>
@@ -1539,7 +1638,7 @@
       <c r="A81" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B81" s="33"/>
+      <c r="B81" s="29"/>
       <c r="C81" s="22">
         <f>SUM(C76:C80)</f>
         <v>0</v>
@@ -1551,7 +1650,7 @@
       <c r="A82" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B82" s="34"/>
+      <c r="B82" s="30"/>
       <c r="C82" s="25"/>
       <c r="D82" s="26"/>
       <c r="E82" s="27"/>
@@ -1560,35 +1659,35 @@
       <c r="A83" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B83" s="32"/>
+      <c r="B83" s="28"/>
       <c r="C83" s="5"/>
       <c r="D83" s="6"/>
       <c r="E83" s="21"/>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A84" s="7"/>
-      <c r="B84" s="33"/>
+      <c r="B84" s="29"/>
       <c r="C84" s="8"/>
       <c r="D84" s="9"/>
       <c r="E84" s="8"/>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A85" s="7"/>
-      <c r="B85" s="33"/>
+      <c r="B85" s="29"/>
       <c r="C85" s="8"/>
       <c r="D85" s="9"/>
       <c r="E85" s="8"/>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A86" s="7"/>
-      <c r="B86" s="33"/>
+      <c r="B86" s="29"/>
       <c r="C86" s="8"/>
       <c r="D86" s="9"/>
       <c r="E86" s="8"/>
     </row>
     <row r="87" spans="1:5" ht="14.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A87" s="10"/>
-      <c r="B87" s="33"/>
+      <c r="B87" s="29"/>
       <c r="C87" s="10"/>
       <c r="D87" s="11"/>
       <c r="E87" s="10"/>
@@ -1597,7 +1696,7 @@
       <c r="A88" s="12" t="s">
         <v>17</v>
       </c>
-      <c r="B88" s="33"/>
+      <c r="B88" s="29"/>
       <c r="C88" s="22">
         <f>SUM(C83:C87)</f>
         <v>0</v>
@@ -1609,19 +1708,19 @@
       <c r="A89" s="12" t="s">
         <v>13</v>
       </c>
-      <c r="B89" s="34"/>
+      <c r="B89" s="30"/>
       <c r="C89" s="25"/>
       <c r="D89" s="26"/>
       <c r="E89" s="27"/>
     </row>
     <row r="90" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A90" s="35" t="s">
+      <c r="A90" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="B90" s="36"/>
+      <c r="B90" s="32"/>
       <c r="C90" s="13">
         <f>MROUND(SUM(C6:C89) /8,0.2)</f>
-        <v>6</v>
+        <v>18</v>
       </c>
       <c r="D90" s="14"/>
       <c r="E90" s="15"/>
@@ -1636,31 +1735,6 @@
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="D81:E81"/>
-    <mergeCell ref="C82:E82"/>
-    <mergeCell ref="B83:B89"/>
-    <mergeCell ref="D88:E88"/>
-    <mergeCell ref="C89:E89"/>
-    <mergeCell ref="D67:E67"/>
-    <mergeCell ref="C68:E68"/>
-    <mergeCell ref="B69:B75"/>
-    <mergeCell ref="D74:E74"/>
-    <mergeCell ref="C75:E75"/>
-    <mergeCell ref="B27:B33"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="C33:E33"/>
-    <mergeCell ref="D53:E53"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="C40:E40"/>
-    <mergeCell ref="D46:E46"/>
-    <mergeCell ref="C47:E47"/>
-    <mergeCell ref="A90:B90"/>
-    <mergeCell ref="B34:B40"/>
-    <mergeCell ref="B41:B47"/>
-    <mergeCell ref="B48:B54"/>
-    <mergeCell ref="B55:B61"/>
-    <mergeCell ref="B62:B68"/>
-    <mergeCell ref="B76:B82"/>
     <mergeCell ref="D60:E60"/>
     <mergeCell ref="C61:E61"/>
     <mergeCell ref="B1:C1"/>
@@ -1677,6 +1751,31 @@
     <mergeCell ref="B20:B26"/>
     <mergeCell ref="D25:E25"/>
     <mergeCell ref="C26:E26"/>
+    <mergeCell ref="A90:B90"/>
+    <mergeCell ref="B34:B40"/>
+    <mergeCell ref="B41:B47"/>
+    <mergeCell ref="B48:B54"/>
+    <mergeCell ref="B55:B61"/>
+    <mergeCell ref="B62:B68"/>
+    <mergeCell ref="B76:B82"/>
+    <mergeCell ref="B27:B33"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="C33:E33"/>
+    <mergeCell ref="D53:E53"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="C40:E40"/>
+    <mergeCell ref="D46:E46"/>
+    <mergeCell ref="C47:E47"/>
+    <mergeCell ref="D67:E67"/>
+    <mergeCell ref="C68:E68"/>
+    <mergeCell ref="B69:B75"/>
+    <mergeCell ref="D74:E74"/>
+    <mergeCell ref="C75:E75"/>
+    <mergeCell ref="D81:E81"/>
+    <mergeCell ref="C82:E82"/>
+    <mergeCell ref="B83:B89"/>
+    <mergeCell ref="D88:E88"/>
+    <mergeCell ref="C89:E89"/>
   </mergeCells>
   <dataValidations count="1">
     <dataValidation type="whole" operator="greaterThan" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Durée par tranche de 10min" error="Le nombre doit être de type entier" sqref="B6 C6:C11 B13 C13:C18 B20 C20:C25 B27 C27:C32 B34 C34:C39 B41 C41:C46 B48 C48:C53 B55 C55:C60 B62 C62:C67 B69 C69:C74 B76 C76:C81 B83 C83:C88" xr:uid="{345ABA8F-B69F-4AFC-9D0E-D2AB0ACDE277}">
@@ -1704,12 +1803,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100FBB99F57F4D89D439F52EDCD0CED316B" ma:contentTypeVersion="7" ma:contentTypeDescription="Crée un document." ma:contentTypeScope="" ma:versionID="d33ce6f53f467230af3a4d19e3409e37">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="6b19550a-bdc3-4796-8096-c6911560d534" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="fd1611c028c4b8e5ae6fe3ffca8b06cf" ns2:_="">
     <xsd:import namespace="6b19550a-bdc3-4796-8096-c6911560d534"/>
@@ -1871,6 +1964,12 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{38BCAAC0-9C03-42D2-8685-2E30F60CCBAA}">
   <ds:schemaRefs>
@@ -1880,15 +1979,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80685F9E-CFF7-4CE8-86AB-E177C421B2C5}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -1904,4 +1994,13 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{80568DEC-920F-4A54-AD30-257A3312E4FF}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>